<commit_message>
rerun model qwen3.5:9b RAG COT Model results generated
</commit_message>
<xml_diff>
--- a/results/qwen3_5_9b/comparison_CoTRAG/CoTRAG_costs.xlsx
+++ b/results/qwen3_5_9b/comparison_CoTRAG/CoTRAG_costs.xlsx
@@ -472,25 +472,25 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1.706821918487549</v>
+        <v>28.14152073860168</v>
       </c>
       <c r="B2" t="n">
-        <v>1420.18359375</v>
+        <v>1423.96484375</v>
       </c>
       <c r="C2" t="n">
-        <v>11.2</v>
+        <v>12.2</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>0.349987268447876</v>
+        <v>0.6831538677215576</v>
       </c>
       <c r="G2" t="n">
-        <v>1.356829881668091</v>
+        <v>27.45836162567139</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -498,25 +498,25 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2.319665908813477</v>
+        <v>15.52196788787842</v>
       </c>
       <c r="B3" t="n">
-        <v>1420.421875</v>
+        <v>1424.18359375</v>
       </c>
       <c r="C3" t="n">
-        <v>8.9</v>
+        <v>14.1</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>0.09566617012023926</v>
+        <v>0.2805397510528564</v>
       </c>
       <c r="G3" t="n">
-        <v>2.223996162414551</v>
+        <v>15.24142456054688</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
@@ -524,25 +524,25 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.7850995063781738</v>
+        <v>12.55752444267273</v>
       </c>
       <c r="B4" t="n">
-        <v>1420.4921875</v>
+        <v>1424.30078125</v>
       </c>
       <c r="C4" t="n">
-        <v>8.4</v>
+        <v>14.3</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>0.09102272987365723</v>
+        <v>0.2421054840087891</v>
       </c>
       <c r="G4" t="n">
-        <v>0.6940741539001465</v>
+        <v>12.31541633605957</v>
       </c>
       <c r="H4" t="n">
         <v>0</v>
@@ -550,25 +550,25 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1.906833410263062</v>
+        <v>13.74409937858582</v>
       </c>
       <c r="B5" t="n">
-        <v>1420.58984375</v>
+        <v>1425.84765625</v>
       </c>
       <c r="C5" t="n">
-        <v>9.5</v>
+        <v>12.5</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>0.08823752403259277</v>
+        <v>0.2770164012908936</v>
       </c>
       <c r="G5" t="n">
-        <v>1.818592548370361</v>
+        <v>13.46707987785339</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
@@ -576,25 +576,25 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>1.474850177764893</v>
+        <v>11.42347955703735</v>
       </c>
       <c r="B6" t="n">
-        <v>1420.6015625</v>
+        <v>1425.9453125</v>
       </c>
       <c r="C6" t="n">
-        <v>8.9</v>
+        <v>14.6</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>0.05181241035461426</v>
+        <v>0.2424299716949463</v>
       </c>
       <c r="G6" t="n">
-        <v>1.423035144805908</v>
+        <v>11.18104696273804</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
@@ -602,25 +602,25 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0.413616418838501</v>
+        <v>30.12495017051697</v>
       </c>
       <c r="B7" t="n">
-        <v>1420.68359375</v>
+        <v>1426.12890625</v>
       </c>
       <c r="C7" t="n">
-        <v>8.800000000000001</v>
+        <v>14.7</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>0.04916119575500488</v>
+        <v>0.2809305191040039</v>
       </c>
       <c r="G7" t="n">
-        <v>0.3644523620605469</v>
+        <v>29.84401655197144</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
@@ -628,25 +628,25 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>2.103248119354248</v>
+        <v>20.1275327205658</v>
       </c>
       <c r="B8" t="n">
-        <v>1420.8125</v>
+        <v>1426.25</v>
       </c>
       <c r="C8" t="n">
-        <v>17.8</v>
+        <v>13.6</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>0.05114030838012695</v>
+        <v>0.278907299041748</v>
       </c>
       <c r="G8" t="n">
-        <v>2.052104711532593</v>
+        <v>19.84862327575684</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
@@ -654,25 +654,25 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0.4237608909606934</v>
+        <v>24.18343162536621</v>
       </c>
       <c r="B9" t="n">
-        <v>1420.8125</v>
+        <v>1426.27734375</v>
       </c>
       <c r="C9" t="n">
-        <v>17.9</v>
+        <v>14.8</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>0.04909753799438477</v>
+        <v>0.2916948795318604</v>
       </c>
       <c r="G9" t="n">
-        <v>0.3746600151062012</v>
+        <v>23.89173412322998</v>
       </c>
       <c r="H9" t="n">
         <v>0</v>
@@ -680,25 +680,25 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>2.480668067932129</v>
+        <v>34.16134881973267</v>
       </c>
       <c r="B10" t="n">
-        <v>1420.89453125</v>
+        <v>1426.40234375</v>
       </c>
       <c r="C10" t="n">
-        <v>12</v>
+        <v>15.1</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>0.120957612991333</v>
+        <v>0.2813558578491211</v>
       </c>
       <c r="G10" t="n">
-        <v>2.359707593917847</v>
+        <v>33.87999033927917</v>
       </c>
       <c r="H10" t="n">
         <v>0</v>
@@ -706,25 +706,25 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>1.657833337783813</v>
+        <v>17.57684969902039</v>
       </c>
       <c r="B11" t="n">
-        <v>1420.99609375</v>
+        <v>1426.50390625</v>
       </c>
       <c r="C11" t="n">
-        <v>9</v>
+        <v>12.6</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>0.04956936836242676</v>
+        <v>0.236943244934082</v>
       </c>
       <c r="G11" t="n">
-        <v>1.608261585235596</v>
+        <v>17.33990359306335</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
@@ -732,25 +732,25 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>1.701315641403198</v>
+        <v>24.72253727912903</v>
       </c>
       <c r="B12" t="n">
-        <v>1421.04296875</v>
+        <v>1426.5234375</v>
       </c>
       <c r="C12" t="n">
-        <v>9.5</v>
+        <v>14.8</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>0.04933333396911621</v>
+        <v>0.2424871921539307</v>
       </c>
       <c r="G12" t="n">
-        <v>1.651979446411133</v>
+        <v>24.48004722595215</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -758,25 +758,25 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>2.509064912796021</v>
+        <v>17.93367052078247</v>
       </c>
       <c r="B13" t="n">
-        <v>1421.11328125</v>
+        <v>1426.52734375</v>
       </c>
       <c r="C13" t="n">
-        <v>9</v>
+        <v>14.6</v>
       </c>
       <c r="D13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>0.05124020576477051</v>
+        <v>0.2536413669586182</v>
       </c>
       <c r="G13" t="n">
-        <v>2.457822322845459</v>
+        <v>17.68002653121948</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -784,25 +784,25 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>1.387258291244507</v>
+        <v>42.45850825309753</v>
       </c>
       <c r="B14" t="n">
-        <v>1421.19921875</v>
+        <v>1426.58984375</v>
       </c>
       <c r="C14" t="n">
-        <v>9</v>
+        <v>14.5</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>0.05224132537841797</v>
+        <v>0.23722243309021</v>
       </c>
       <c r="G14" t="n">
-        <v>1.335014581680298</v>
+        <v>42.22128295898438</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -810,25 +810,25 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>2.518002033233643</v>
+        <v>21.11018228530884</v>
       </c>
       <c r="B15" t="n">
-        <v>1421.24609375</v>
+        <v>1426.671875</v>
       </c>
       <c r="C15" t="n">
-        <v>15.3</v>
+        <v>14.8</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>0.05099248886108398</v>
+        <v>0.2437012195587158</v>
       </c>
       <c r="G15" t="n">
-        <v>2.467007398605347</v>
+        <v>20.86647796630859</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -836,25 +836,25 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>1.026593208312988</v>
+        <v>31.17437195777893</v>
       </c>
       <c r="B16" t="n">
-        <v>1421.24609375</v>
+        <v>1426.703125</v>
       </c>
       <c r="C16" t="n">
-        <v>18.4</v>
+        <v>14.7</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>0.05089664459228516</v>
+        <v>0.2448248863220215</v>
       </c>
       <c r="G16" t="n">
-        <v>0.9756934642791748</v>
+        <v>30.92954397201538</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -862,25 +862,25 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>1.281811714172363</v>
+        <v>45.16979837417603</v>
       </c>
       <c r="B17" t="n">
-        <v>1421.24609375</v>
+        <v>1426.796875</v>
       </c>
       <c r="C17" t="n">
-        <v>11.3</v>
+        <v>14.6</v>
       </c>
       <c r="D17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>0.05534815788269043</v>
+        <v>0.2408351898193359</v>
       </c>
       <c r="G17" t="n">
-        <v>1.226461172103882</v>
+        <v>44.92896103858948</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -888,25 +888,25 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>1.795159578323364</v>
+        <v>30.74105763435364</v>
       </c>
       <c r="B18" t="n">
-        <v>1421.25</v>
+        <v>1426.875</v>
       </c>
       <c r="C18" t="n">
-        <v>9</v>
+        <v>14.6</v>
       </c>
       <c r="D18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>0.04862594604492188</v>
+        <v>0.2813055515289307</v>
       </c>
       <c r="G18" t="n">
-        <v>1.746531009674072</v>
+        <v>30.4597499370575</v>
       </c>
       <c r="H18" t="n">
         <v>0</v>
@@ -914,25 +914,25 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>0.4386868476867676</v>
+        <v>16.41390299797058</v>
       </c>
       <c r="B19" t="n">
-        <v>1421.328125</v>
+        <v>1426.9453125</v>
       </c>
       <c r="C19" t="n">
-        <v>9.300000000000001</v>
+        <v>14.1</v>
       </c>
       <c r="D19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>0.04829859733581543</v>
+        <v>0.2434377670288086</v>
       </c>
       <c r="G19" t="n">
-        <v>0.3903858661651611</v>
+        <v>16.1704626083374</v>
       </c>
       <c r="H19" t="n">
         <v>0</v>
@@ -940,25 +940,25 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>1.664188623428345</v>
+        <v>18.79751110076904</v>
       </c>
       <c r="B20" t="n">
-        <v>1421.3359375</v>
+        <v>1427.02734375</v>
       </c>
       <c r="C20" t="n">
-        <v>9.1</v>
+        <v>13.3</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>0.04989814758300781</v>
+        <v>0.2724058628082275</v>
       </c>
       <c r="G20" t="n">
-        <v>1.614287853240967</v>
+        <v>18.52510261535645</v>
       </c>
       <c r="H20" t="n">
         <v>0</v>
@@ -966,25 +966,25 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>0.6557137966156006</v>
+        <v>120.5542068481445</v>
       </c>
       <c r="B21" t="n">
-        <v>1421.60546875</v>
+        <v>1427.18359375</v>
       </c>
       <c r="C21" t="n">
-        <v>9.1</v>
+        <v>15</v>
       </c>
       <c r="D21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>0.05228066444396973</v>
+        <v>0.3165504932403564</v>
       </c>
       <c r="G21" t="n">
-        <v>0.6034309864044189</v>
+        <v>120.2376534938812</v>
       </c>
       <c r="H21" t="n">
         <v>0</v>
@@ -992,25 +992,25 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>1.696043014526367</v>
+        <v>23.7665798664093</v>
       </c>
       <c r="B22" t="n">
-        <v>1421.6640625</v>
+        <v>1427.21484375</v>
       </c>
       <c r="C22" t="n">
-        <v>9.199999999999999</v>
+        <v>14.3</v>
       </c>
       <c r="D22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>0.04996848106384277</v>
+        <v>1.423193454742432</v>
       </c>
       <c r="G22" t="n">
-        <v>1.646071910858154</v>
+        <v>22.3433837890625</v>
       </c>
       <c r="H22" t="n">
         <v>0</v>
@@ -1018,25 +1018,25 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>1.673414468765259</v>
+        <v>20.15850138664246</v>
       </c>
       <c r="B23" t="n">
-        <v>1421.6796875</v>
+        <v>1427.23046875</v>
       </c>
       <c r="C23" t="n">
-        <v>8.9</v>
+        <v>13.8</v>
       </c>
       <c r="D23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>0.0524594783782959</v>
+        <v>0.2364990711212158</v>
       </c>
       <c r="G23" t="n">
-        <v>1.620952844619751</v>
+        <v>19.92199993133545</v>
       </c>
       <c r="H23" t="n">
         <v>0</v>
@@ -1044,25 +1044,25 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>1.170245409011841</v>
+        <v>18.35392165184021</v>
       </c>
       <c r="B24" t="n">
-        <v>1421.75</v>
+        <v>1427.2890625</v>
       </c>
       <c r="C24" t="n">
-        <v>10.4</v>
+        <v>13.9</v>
       </c>
       <c r="D24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>0.04999351501464844</v>
+        <v>0.2829515933990479</v>
       </c>
       <c r="G24" t="n">
-        <v>1.12024998664856</v>
+        <v>18.07096767425537</v>
       </c>
       <c r="H24" t="n">
         <v>0</v>
@@ -1070,25 +1070,25 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>1.458403587341309</v>
+        <v>9.765125513076782</v>
       </c>
       <c r="B25" t="n">
-        <v>1421.75390625</v>
+        <v>1427.31640625</v>
       </c>
       <c r="C25" t="n">
-        <v>18.6</v>
+        <v>15.1</v>
       </c>
       <c r="D25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>0.04906821250915527</v>
+        <v>0.240358829498291</v>
       </c>
       <c r="G25" t="n">
-        <v>1.409332752227783</v>
+        <v>9.524764537811279</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1096,25 +1096,25 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>1.465075492858887</v>
+        <v>11.67943692207336</v>
       </c>
       <c r="B26" t="n">
-        <v>1421.75390625</v>
+        <v>1427.31640625</v>
       </c>
       <c r="C26" t="n">
-        <v>18.6</v>
+        <v>12.6</v>
       </c>
       <c r="D26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E26" t="n">
         <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>0.05169343948364258</v>
+        <v>0.2349963188171387</v>
       </c>
       <c r="G26" t="n">
-        <v>1.413379430770874</v>
+        <v>11.44443774223328</v>
       </c>
       <c r="H26" t="n">
         <v>0</v>
@@ -1122,25 +1122,25 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>1.524911165237427</v>
+        <v>11.11807060241699</v>
       </c>
       <c r="B27" t="n">
-        <v>1421.7578125</v>
+        <v>1427.37109375</v>
       </c>
       <c r="C27" t="n">
-        <v>8.800000000000001</v>
+        <v>15</v>
       </c>
       <c r="D27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>0.09921360015869141</v>
+        <v>0.2414374351501465</v>
       </c>
       <c r="G27" t="n">
-        <v>1.425694942474365</v>
+        <v>10.8766303062439</v>
       </c>
       <c r="H27" t="n">
         <v>0</v>
@@ -1148,25 +1148,25 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>0.510322093963623</v>
+        <v>11.24601626396179</v>
       </c>
       <c r="B28" t="n">
-        <v>1421.76171875</v>
+        <v>1427.40625</v>
       </c>
       <c r="C28" t="n">
-        <v>8.9</v>
+        <v>14.5</v>
       </c>
       <c r="D28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>0.04949498176574707</v>
+        <v>0.2954463958740234</v>
       </c>
       <c r="G28" t="n">
-        <v>0.4608244895935059</v>
+        <v>10.9505672454834</v>
       </c>
       <c r="H28" t="n">
         <v>0</v>
@@ -1174,25 +1174,25 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>1.419867753982544</v>
+        <v>14.36031126976013</v>
       </c>
       <c r="B29" t="n">
-        <v>1421.77734375</v>
+        <v>1427.48046875</v>
       </c>
       <c r="C29" t="n">
-        <v>9.300000000000001</v>
+        <v>12.7</v>
       </c>
       <c r="D29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E29" t="n">
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>0.04925251007080078</v>
+        <v>0.2365856170654297</v>
       </c>
       <c r="G29" t="n">
-        <v>1.370613574981689</v>
+        <v>14.12372279167175</v>
       </c>
       <c r="H29" t="n">
         <v>0</v>
@@ -1200,25 +1200,25 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>1.292150735855103</v>
+        <v>12.9955415725708</v>
       </c>
       <c r="B30" t="n">
-        <v>1421.7890625</v>
+        <v>1427.52734375</v>
       </c>
       <c r="C30" t="n">
-        <v>8.9</v>
+        <v>14.4</v>
       </c>
       <c r="D30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E30" t="n">
         <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>0.04937362670898438</v>
+        <v>0.2415950298309326</v>
       </c>
       <c r="G30" t="n">
-        <v>1.24277400970459</v>
+        <v>12.75394439697266</v>
       </c>
       <c r="H30" t="n">
         <v>0</v>
@@ -1226,25 +1226,25 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>2.377240419387817</v>
+        <v>23.65238189697266</v>
       </c>
       <c r="B31" t="n">
-        <v>1421.81640625</v>
+        <v>1427.54296875</v>
       </c>
       <c r="C31" t="n">
-        <v>8.6</v>
+        <v>14.9</v>
       </c>
       <c r="D31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E31" t="n">
         <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>0.1925017833709717</v>
+        <v>0.2395443916320801</v>
       </c>
       <c r="G31" t="n">
-        <v>2.184736013412476</v>
+        <v>23.41283512115479</v>
       </c>
       <c r="H31" t="n">
         <v>0</v>
@@ -1252,25 +1252,25 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>1.714750528335571</v>
+        <v>13.19795632362366</v>
       </c>
       <c r="B32" t="n">
-        <v>1421.82421875</v>
+        <v>1427.54296875</v>
       </c>
       <c r="C32" t="n">
-        <v>9.199999999999999</v>
+        <v>12.6</v>
       </c>
       <c r="D32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E32" t="n">
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>0.05134940147399902</v>
+        <v>0.2682473659515381</v>
       </c>
       <c r="G32" t="n">
-        <v>1.663398742675781</v>
+        <v>12.92970585823059</v>
       </c>
       <c r="H32" t="n">
         <v>0</v>
@@ -1278,25 +1278,25 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>1.115107536315918</v>
+        <v>24.24566864967346</v>
       </c>
       <c r="B33" t="n">
-        <v>1421.95703125</v>
+        <v>1427.5625</v>
       </c>
       <c r="C33" t="n">
-        <v>10.4</v>
+        <v>14.9</v>
       </c>
       <c r="D33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E33" t="n">
         <v>0</v>
       </c>
       <c r="F33" t="n">
-        <v>0.0502772331237793</v>
+        <v>0.2397534847259521</v>
       </c>
       <c r="G33" t="n">
-        <v>1.064826726913452</v>
+        <v>24.00591349601746</v>
       </c>
       <c r="H33" t="n">
         <v>0</v>
@@ -1304,25 +1304,25 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>1.966100215911865</v>
+        <v>17.30383276939392</v>
       </c>
       <c r="B34" t="n">
-        <v>1422.01171875</v>
+        <v>1427.5703125</v>
       </c>
       <c r="C34" t="n">
-        <v>18.4</v>
+        <v>14</v>
       </c>
       <c r="D34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E34" t="n">
         <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>0.05168390274047852</v>
+        <v>0.2415008544921875</v>
       </c>
       <c r="G34" t="n">
-        <v>1.914413690567017</v>
+        <v>17.06232929229736</v>
       </c>
       <c r="H34" t="n">
         <v>0</v>
@@ -1330,25 +1330,25 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>0.8537487983703613</v>
+        <v>30.63400864601135</v>
       </c>
       <c r="B35" t="n">
-        <v>1422.0234375</v>
+        <v>1427.64453125</v>
       </c>
       <c r="C35" t="n">
-        <v>18.9</v>
+        <v>14.5</v>
       </c>
       <c r="D35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E35" t="n">
         <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>0.05187606811523438</v>
+        <v>0.2347116470336914</v>
       </c>
       <c r="G35" t="n">
-        <v>0.8018703460693359</v>
+        <v>30.39929342269897</v>
       </c>
       <c r="H35" t="n">
         <v>0</v>
@@ -1356,25 +1356,25 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>1.162926197052002</v>
+        <v>19.29005217552185</v>
       </c>
       <c r="B36" t="n">
-        <v>1422.046875</v>
+        <v>1427.671875</v>
       </c>
       <c r="C36" t="n">
-        <v>9.199999999999999</v>
+        <v>13.9</v>
       </c>
       <c r="D36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E36" t="n">
         <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>0.05158853530883789</v>
+        <v>0.2424337863922119</v>
       </c>
       <c r="G36" t="n">
-        <v>1.111335039138794</v>
+        <v>19.04761600494385</v>
       </c>
       <c r="H36" t="n">
         <v>0</v>
@@ -1382,25 +1382,25 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>2.302383422851562</v>
+        <v>38.33541822433472</v>
       </c>
       <c r="B37" t="n">
-        <v>1422.0625</v>
+        <v>1427.78125</v>
       </c>
       <c r="C37" t="n">
-        <v>9</v>
+        <v>14.9</v>
       </c>
       <c r="D37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E37" t="n">
         <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>0.04957008361816406</v>
+        <v>0.2810478210449219</v>
       </c>
       <c r="G37" t="n">
-        <v>2.252810955047607</v>
+        <v>38.05436754226685</v>
       </c>
       <c r="H37" t="n">
         <v>0</v>
@@ -1408,25 +1408,25 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>1.948634624481201</v>
+        <v>29.98873829841614</v>
       </c>
       <c r="B38" t="n">
-        <v>1422.14453125</v>
+        <v>1427.79296875</v>
       </c>
       <c r="C38" t="n">
-        <v>9.300000000000001</v>
+        <v>14.5</v>
       </c>
       <c r="D38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E38" t="n">
         <v>0</v>
       </c>
       <c r="F38" t="n">
-        <v>0.04948115348815918</v>
+        <v>0.2354922294616699</v>
       </c>
       <c r="G38" t="n">
-        <v>1.899151086807251</v>
+        <v>29.75324296951294</v>
       </c>
       <c r="H38" t="n">
         <v>0</v>
@@ -1434,25 +1434,25 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>1.577873945236206</v>
+        <v>23.14711952209473</v>
       </c>
       <c r="B39" t="n">
-        <v>1422.1484375</v>
+        <v>1427.82421875</v>
       </c>
       <c r="C39" t="n">
-        <v>9.199999999999999</v>
+        <v>14.1</v>
       </c>
       <c r="D39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E39" t="n">
         <v>0</v>
       </c>
       <c r="F39" t="n">
-        <v>0.04948902130126953</v>
+        <v>0.241112232208252</v>
       </c>
       <c r="G39" t="n">
-        <v>1.528383255004883</v>
+        <v>22.9060046672821</v>
       </c>
       <c r="H39" t="n">
         <v>0</v>
@@ -1460,25 +1460,25 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>0.5440893173217773</v>
+        <v>12.27740526199341</v>
       </c>
       <c r="B40" t="n">
-        <v>1422.16015625</v>
+        <v>1427.88671875</v>
       </c>
       <c r="C40" t="n">
-        <v>8.9</v>
+        <v>14</v>
       </c>
       <c r="D40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E40" t="n">
         <v>0</v>
       </c>
       <c r="F40" t="n">
-        <v>0.04987859725952148</v>
+        <v>0.2815837860107422</v>
       </c>
       <c r="G40" t="n">
-        <v>0.4942085742950439</v>
+        <v>11.9958188533783</v>
       </c>
       <c r="H40" t="n">
         <v>0</v>
@@ -1486,25 +1486,25 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>1.611111640930176</v>
+        <v>12.31471705436707</v>
       </c>
       <c r="B41" t="n">
-        <v>1422.16015625</v>
+        <v>1427.91015625</v>
       </c>
       <c r="C41" t="n">
-        <v>9.199999999999999</v>
+        <v>13.6</v>
       </c>
       <c r="D41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E41" t="n">
         <v>0</v>
       </c>
       <c r="F41" t="n">
-        <v>0.04964447021484375</v>
+        <v>0.2349236011505127</v>
       </c>
       <c r="G41" t="n">
-        <v>1.561464786529541</v>
+        <v>12.07979106903076</v>
       </c>
       <c r="H41" t="n">
         <v>0</v>
@@ -1512,25 +1512,25 @@
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>2.062058925628662</v>
+        <v>15.83804440498352</v>
       </c>
       <c r="B42" t="n">
-        <v>1422.21484375</v>
+        <v>1427.9140625</v>
       </c>
       <c r="C42" t="n">
-        <v>14.5</v>
+        <v>15</v>
       </c>
       <c r="D42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E42" t="n">
         <v>0</v>
       </c>
       <c r="F42" t="n">
-        <v>0.0497279167175293</v>
+        <v>0.2399337291717529</v>
       </c>
       <c r="G42" t="n">
-        <v>2.012328147888184</v>
+        <v>15.59810781478882</v>
       </c>
       <c r="H42" t="n">
         <v>0</v>
@@ -1538,25 +1538,25 @@
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>1.796472787857056</v>
+        <v>16.69436430931091</v>
       </c>
       <c r="B43" t="n">
-        <v>1422.296875</v>
+        <v>1427.91796875</v>
       </c>
       <c r="C43" t="n">
-        <v>18.4</v>
+        <v>14.2</v>
       </c>
       <c r="D43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E43" t="n">
         <v>0</v>
       </c>
       <c r="F43" t="n">
-        <v>0.05265164375305176</v>
+        <v>0.2610995769500732</v>
       </c>
       <c r="G43" t="n">
-        <v>1.743818759918213</v>
+        <v>16.43326163291931</v>
       </c>
       <c r="H43" t="n">
         <v>0</v>
@@ -1564,25 +1564,25 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>0.4024243354797363</v>
+        <v>35.15044331550598</v>
       </c>
       <c r="B44" t="n">
-        <v>1422.37890625</v>
+        <v>1427.96484375</v>
       </c>
       <c r="C44" t="n">
-        <v>9.1</v>
+        <v>14.3</v>
       </c>
       <c r="D44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E44" t="n">
         <v>0</v>
       </c>
       <c r="F44" t="n">
-        <v>0.05441999435424805</v>
+        <v>0.2733922004699707</v>
       </c>
       <c r="G44" t="n">
-        <v>0.3480007648468018</v>
+        <v>34.87704825401306</v>
       </c>
       <c r="H44" t="n">
         <v>0</v>
@@ -1590,25 +1590,25 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>1.285399675369263</v>
+        <v>51.59527850151062</v>
       </c>
       <c r="B45" t="n">
-        <v>1422.40625</v>
+        <v>1428.03515625</v>
       </c>
       <c r="C45" t="n">
-        <v>8.9</v>
+        <v>14.9</v>
       </c>
       <c r="D45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E45" t="n">
         <v>0</v>
       </c>
       <c r="F45" t="n">
-        <v>0.04978108406066895</v>
+        <v>0.240816593170166</v>
       </c>
       <c r="G45" t="n">
-        <v>1.235615253448486</v>
+        <v>51.35445880889893</v>
       </c>
       <c r="H45" t="n">
         <v>0</v>
@@ -1616,25 +1616,25 @@
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>1.114473581314087</v>
+        <v>23.64381003379822</v>
       </c>
       <c r="B46" t="n">
-        <v>1422.4140625</v>
+        <v>1428.10546875</v>
       </c>
       <c r="C46" t="n">
-        <v>9</v>
+        <v>14.8</v>
       </c>
       <c r="D46" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E46" t="n">
         <v>0</v>
       </c>
       <c r="F46" t="n">
-        <v>0.04797625541687012</v>
+        <v>0.2393677234649658</v>
       </c>
       <c r="G46" t="n">
-        <v>1.066495180130005</v>
+        <v>23.40443968772888</v>
       </c>
       <c r="H46" t="n">
         <v>0</v>
@@ -1642,25 +1642,25 @@
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>1.099425077438354</v>
+        <v>29.54692220687866</v>
       </c>
       <c r="B47" t="n">
-        <v>1422.43359375</v>
+        <v>1428.20703125</v>
       </c>
       <c r="C47" t="n">
-        <v>9.699999999999999</v>
+        <v>13.6</v>
       </c>
       <c r="D47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E47" t="n">
         <v>0</v>
       </c>
       <c r="F47" t="n">
-        <v>0.05115509033203125</v>
+        <v>0.241060733795166</v>
       </c>
       <c r="G47" t="n">
-        <v>1.048267602920532</v>
+        <v>29.30585932731628</v>
       </c>
       <c r="H47" t="n">
         <v>0</v>
@@ -1668,25 +1668,25 @@
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>2.222482442855835</v>
+        <v>26.36601758003235</v>
       </c>
       <c r="B48" t="n">
-        <v>1422.44140625</v>
+        <v>1428.2578125</v>
       </c>
       <c r="C48" t="n">
-        <v>9.300000000000001</v>
+        <v>14.7</v>
       </c>
       <c r="D48" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E48" t="n">
         <v>0</v>
       </c>
       <c r="F48" t="n">
-        <v>0.0501246452331543</v>
+        <v>0.241774320602417</v>
       </c>
       <c r="G48" t="n">
-        <v>2.172355651855469</v>
+        <v>26.12423872947693</v>
       </c>
       <c r="H48" t="n">
         <v>0</v>
@@ -1694,25 +1694,25 @@
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>0.8767650127410889</v>
+        <v>25.7324275970459</v>
       </c>
       <c r="B49" t="n">
-        <v>1422.515625</v>
+        <v>1428.2734375</v>
       </c>
       <c r="C49" t="n">
-        <v>8.4</v>
+        <v>14.8</v>
       </c>
       <c r="D49" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E49" t="n">
         <v>0</v>
       </c>
       <c r="F49" t="n">
-        <v>0.1152732372283936</v>
+        <v>0.2490670680999756</v>
       </c>
       <c r="G49" t="n">
-        <v>0.7614893913269043</v>
+        <v>25.48335790634155</v>
       </c>
       <c r="H49" t="n">
         <v>0</v>
@@ -1720,25 +1720,25 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>1.342483520507812</v>
+        <v>32.11345148086548</v>
       </c>
       <c r="B50" t="n">
-        <v>1422.515625</v>
+        <v>1428.328125</v>
       </c>
       <c r="C50" t="n">
-        <v>10</v>
+        <v>14.4</v>
       </c>
       <c r="D50" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E50" t="n">
         <v>0</v>
       </c>
       <c r="F50" t="n">
-        <v>0.04998922348022461</v>
+        <v>0.2362794876098633</v>
       </c>
       <c r="G50" t="n">
-        <v>1.292491912841797</v>
+        <v>31.87716865539551</v>
       </c>
       <c r="H50" t="n">
         <v>0</v>
@@ -1746,25 +1746,25 @@
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>1.789185047149658</v>
+        <v>38.95255517959595</v>
       </c>
       <c r="B51" t="n">
-        <v>1422.55859375</v>
+        <v>1428.3828125</v>
       </c>
       <c r="C51" t="n">
-        <v>10.2</v>
+        <v>14.8</v>
       </c>
       <c r="D51" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E51" t="n">
         <v>0</v>
       </c>
       <c r="F51" t="n">
-        <v>0.05191898345947266</v>
+        <v>0.2860369682312012</v>
       </c>
       <c r="G51" t="n">
-        <v>1.737263441085815</v>
+        <v>38.66651153564453</v>
       </c>
       <c r="H51" t="n">
         <v>0</v>
@@ -1772,25 +1772,25 @@
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>1.112174272537231</v>
+        <v>22.05804204940796</v>
       </c>
       <c r="B52" t="n">
-        <v>1422.625</v>
+        <v>1428.390625</v>
       </c>
       <c r="C52" t="n">
-        <v>18.3</v>
+        <v>14.4</v>
       </c>
       <c r="D52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E52" t="n">
         <v>0</v>
       </c>
       <c r="F52" t="n">
-        <v>0.05055522918701172</v>
+        <v>0.2756595611572266</v>
       </c>
       <c r="G52" t="n">
-        <v>1.061616897583008</v>
+        <v>21.78237915039062</v>
       </c>
       <c r="H52" t="n">
         <v>0</v>
@@ -1798,25 +1798,25 @@
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>1.710916757583618</v>
+        <v>23.49525189399719</v>
       </c>
       <c r="B53" t="n">
-        <v>1422.765625</v>
+        <v>1428.40234375</v>
       </c>
       <c r="C53" t="n">
-        <v>18.7</v>
+        <v>13.5</v>
       </c>
       <c r="D53" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E53" t="n">
         <v>0</v>
       </c>
       <c r="F53" t="n">
-        <v>0.0487210750579834</v>
+        <v>0.2365756034851074</v>
       </c>
       <c r="G53" t="n">
-        <v>1.662192821502686</v>
+        <v>23.25867247581482</v>
       </c>
       <c r="H53" t="n">
         <v>0</v>
@@ -1824,25 +1824,25 @@
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>1.957052707672119</v>
+        <v>18.25840330123901</v>
       </c>
       <c r="B54" t="n">
-        <v>1422.7890625</v>
+        <v>1428.44921875</v>
       </c>
       <c r="C54" t="n">
-        <v>9.5</v>
+        <v>14.9</v>
       </c>
       <c r="D54" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E54" t="n">
         <v>0</v>
       </c>
       <c r="F54" t="n">
-        <v>0.04836034774780273</v>
+        <v>0.2397184371948242</v>
       </c>
       <c r="G54" t="n">
-        <v>1.908689498901367</v>
+        <v>18.0186824798584</v>
       </c>
       <c r="H54" t="n">
         <v>0</v>
@@ -1850,25 +1850,25 @@
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>0.4313206672668457</v>
+        <v>24.1825840473175</v>
       </c>
       <c r="B55" t="n">
-        <v>1422.79296875</v>
+        <v>1428.44921875</v>
       </c>
       <c r="C55" t="n">
-        <v>8.699999999999999</v>
+        <v>14.9</v>
       </c>
       <c r="D55" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E55" t="n">
         <v>0</v>
       </c>
       <c r="F55" t="n">
-        <v>0.04838085174560547</v>
+        <v>0.2392697334289551</v>
       </c>
       <c r="G55" t="n">
-        <v>0.3829376697540283</v>
+        <v>23.94331240653992</v>
       </c>
       <c r="H55" t="n">
         <v>0</v>
@@ -1876,25 +1876,25 @@
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>1.150134563446045</v>
+        <v>28.07696628570557</v>
       </c>
       <c r="B56" t="n">
-        <v>1422.79296875</v>
+        <v>1428.453125</v>
       </c>
       <c r="C56" t="n">
-        <v>9</v>
+        <v>13.6</v>
       </c>
       <c r="D56" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E56" t="n">
         <v>0</v>
       </c>
       <c r="F56" t="n">
-        <v>0.04962730407714844</v>
+        <v>0.2880773544311523</v>
       </c>
       <c r="G56" t="n">
-        <v>1.100505352020264</v>
+        <v>27.78888702392578</v>
       </c>
       <c r="H56" t="n">
         <v>0</v>
@@ -1902,25 +1902,25 @@
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>0.4090378284454346</v>
+        <v>22.16571664810181</v>
       </c>
       <c r="B57" t="n">
-        <v>1422.796875</v>
+        <v>1428.57421875</v>
       </c>
       <c r="C57" t="n">
-        <v>9.199999999999999</v>
+        <v>14.9</v>
       </c>
       <c r="D57" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E57" t="n">
         <v>0</v>
       </c>
       <c r="F57" t="n">
-        <v>0.05159854888916016</v>
+        <v>0.2532205581665039</v>
       </c>
       <c r="G57" t="n">
-        <v>0.3574364185333252</v>
+        <v>21.91249418258667</v>
       </c>
       <c r="H57" t="n">
         <v>0</v>
@@ -1928,25 +1928,25 @@
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>1.964935064315796</v>
+        <v>14.46353507041931</v>
       </c>
       <c r="B58" t="n">
-        <v>1422.8125</v>
+        <v>1428.65625</v>
       </c>
       <c r="C58" t="n">
-        <v>9.300000000000001</v>
+        <v>14.2</v>
       </c>
       <c r="D58" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E58" t="n">
         <v>0</v>
       </c>
       <c r="F58" t="n">
-        <v>0.05034136772155762</v>
+        <v>0.2409212589263916</v>
       </c>
       <c r="G58" t="n">
-        <v>1.91459059715271</v>
+        <v>14.22261095046997</v>
       </c>
       <c r="H58" t="n">
         <v>0</v>
@@ -1954,25 +1954,25 @@
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>0.514394998550415</v>
+        <v>15.82165861129761</v>
       </c>
       <c r="B59" t="n">
-        <v>1422.84765625</v>
+        <v>1428.75</v>
       </c>
       <c r="C59" t="n">
-        <v>8.6</v>
+        <v>12.6</v>
       </c>
       <c r="D59" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E59" t="n">
         <v>0</v>
       </c>
       <c r="F59" t="n">
-        <v>0.05374026298522949</v>
+        <v>0.2703752517700195</v>
       </c>
       <c r="G59" t="n">
-        <v>0.4606523513793945</v>
+        <v>15.55128026008606</v>
       </c>
       <c r="H59" t="n">
         <v>0</v>
@@ -1980,25 +1980,25 @@
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>1.0070481300354</v>
+        <v>19.068115234375</v>
       </c>
       <c r="B60" t="n">
-        <v>1422.8828125</v>
+        <v>1428.828125</v>
       </c>
       <c r="C60" t="n">
-        <v>8.800000000000001</v>
+        <v>15.4</v>
       </c>
       <c r="D60" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E60" t="n">
         <v>0</v>
       </c>
       <c r="F60" t="n">
-        <v>0.05050301551818848</v>
+        <v>0.2418711185455322</v>
       </c>
       <c r="G60" t="n">
-        <v>0.9565427303314209</v>
+        <v>18.82624125480652</v>
       </c>
       <c r="H60" t="n">
         <v>0</v>
@@ -2006,25 +2006,25 @@
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>1.330243349075317</v>
+        <v>23.78583002090454</v>
       </c>
       <c r="B61" t="n">
-        <v>1422.8984375</v>
+        <v>1428.8359375</v>
       </c>
       <c r="C61" t="n">
-        <v>9.1</v>
+        <v>14.9</v>
       </c>
       <c r="D61" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E61" t="n">
         <v>0</v>
       </c>
       <c r="F61" t="n">
-        <v>0.04955029487609863</v>
+        <v>0.2427754402160645</v>
       </c>
       <c r="G61" t="n">
-        <v>1.280691146850586</v>
+        <v>23.54305171966553</v>
       </c>
       <c r="H61" t="n">
         <v>0</v>
@@ -2032,25 +2032,25 @@
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>1.064628839492798</v>
+        <v>19.27034783363342</v>
       </c>
       <c r="B62" t="n">
-        <v>1422.91015625</v>
+        <v>1428.8359375</v>
       </c>
       <c r="C62" t="n">
-        <v>9.5</v>
+        <v>12.7</v>
       </c>
       <c r="D62" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E62" t="n">
         <v>0</v>
       </c>
       <c r="F62" t="n">
-        <v>0.0484459400177002</v>
+        <v>0.2710907459259033</v>
       </c>
       <c r="G62" t="n">
-        <v>1.016180276870728</v>
+        <v>18.99925470352173</v>
       </c>
       <c r="H62" t="n">
         <v>0</v>
@@ -2058,25 +2058,25 @@
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>0.5330078601837158</v>
+        <v>20.45079207420349</v>
       </c>
       <c r="B63" t="n">
-        <v>1422.96484375</v>
+        <v>1428.8359375</v>
       </c>
       <c r="C63" t="n">
-        <v>15.8</v>
+        <v>15.3</v>
       </c>
       <c r="D63" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E63" t="n">
         <v>0</v>
       </c>
       <c r="F63" t="n">
-        <v>0.0521705150604248</v>
+        <v>0.2729942798614502</v>
       </c>
       <c r="G63" t="n">
-        <v>0.4808344841003418</v>
+        <v>20.17779445648193</v>
       </c>
       <c r="H63" t="n">
         <v>0</v>
@@ -2084,25 +2084,25 @@
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>0.6343700885772705</v>
+        <v>27.08725309371948</v>
       </c>
       <c r="B64" t="n">
-        <v>1423.01171875</v>
+        <v>1428.8359375</v>
       </c>
       <c r="C64" t="n">
-        <v>18.4</v>
+        <v>14.7</v>
       </c>
       <c r="D64" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E64" t="n">
         <v>0</v>
       </c>
       <c r="F64" t="n">
-        <v>0.0495448112487793</v>
+        <v>0.2595696449279785</v>
       </c>
       <c r="G64" t="n">
-        <v>0.5848231315612793</v>
+        <v>26.82768082618713</v>
       </c>
       <c r="H64" t="n">
         <v>0</v>
@@ -2110,25 +2110,25 @@
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>0.5355420112609863</v>
+        <v>17.49422287940979</v>
       </c>
       <c r="B65" t="n">
-        <v>1423.03125</v>
+        <v>1428.8359375</v>
       </c>
       <c r="C65" t="n">
-        <v>18.3</v>
+        <v>13</v>
       </c>
       <c r="D65" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E65" t="n">
         <v>0</v>
       </c>
       <c r="F65" t="n">
-        <v>0.05477666854858398</v>
+        <v>0.2382171154022217</v>
       </c>
       <c r="G65" t="n">
-        <v>0.4807629585266113</v>
+        <v>17.25600385665894</v>
       </c>
       <c r="H65" t="n">
         <v>0</v>
@@ -2136,25 +2136,25 @@
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>1.633043050765991</v>
+        <v>26.71403932571411</v>
       </c>
       <c r="B66" t="n">
-        <v>1423.03515625</v>
+        <v>1428.8359375</v>
       </c>
       <c r="C66" t="n">
-        <v>17.7</v>
+        <v>14.9</v>
       </c>
       <c r="D66" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E66" t="n">
         <v>0</v>
       </c>
       <c r="F66" t="n">
-        <v>0.0508263111114502</v>
+        <v>0.2412741184234619</v>
       </c>
       <c r="G66" t="n">
-        <v>1.582214593887329</v>
+        <v>26.4727623462677</v>
       </c>
       <c r="H66" t="n">
         <v>0</v>
@@ -2162,25 +2162,25 @@
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>1.263818025588989</v>
+        <v>31.29414844512939</v>
       </c>
       <c r="B67" t="n">
-        <v>1423.0390625</v>
+        <v>1428.87890625</v>
       </c>
       <c r="C67" t="n">
-        <v>9</v>
+        <v>14.7</v>
       </c>
       <c r="D67" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E67" t="n">
         <v>0</v>
       </c>
       <c r="F67" t="n">
-        <v>0.05042791366577148</v>
+        <v>0.2420082092285156</v>
       </c>
       <c r="G67" t="n">
-        <v>1.213387727737427</v>
+        <v>31.05213713645935</v>
       </c>
       <c r="H67" t="n">
         <v>0</v>
@@ -2188,25 +2188,25 @@
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>0.4204361438751221</v>
+        <v>54.51508378982544</v>
       </c>
       <c r="B68" t="n">
-        <v>1423.05078125</v>
+        <v>1428.9765625</v>
       </c>
       <c r="C68" t="n">
-        <v>8.699999999999999</v>
+        <v>14.3</v>
       </c>
       <c r="D68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E68" t="n">
         <v>0</v>
       </c>
       <c r="F68" t="n">
-        <v>0.04936838150024414</v>
+        <v>0.2401511669158936</v>
       </c>
       <c r="G68" t="n">
-        <v>0.3710649013519287</v>
+        <v>54.2749297618866</v>
       </c>
       <c r="H68" t="n">
         <v>0</v>

</xml_diff>